<commit_message>
Deployed 6b3bd1b with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/facturas/API-Emision_ARG-Factura_E.xlsx
+++ b/facturas/API-Emision_ARG-Factura_E.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e420987b8cd2baf4/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gp21263\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="186" documentId="11_C70C9A53E5F1CB35E2F30DB4C40320E0654C3091" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A9D35F0-8E77-446C-BCC6-50631A761DB0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Página1" sheetId="1" r:id="rId1"/>
@@ -1096,19 +1096,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H59"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="4.140625" customWidth="1"/>
-    <col min="4" max="4" width="54.85546875" customWidth="1"/>
-    <col min="5" max="5" width="3.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.85546875" customWidth="1"/>
-    <col min="8" max="8" width="94.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" customWidth="1"/>
+    <col min="3" max="3" width="4.109375" customWidth="1"/>
+    <col min="4" max="4" width="54.88671875" customWidth="1"/>
+    <col min="5" max="5" width="3.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.88671875" customWidth="1"/>
+    <col min="8" max="8" width="94.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1120,7 @@
       <c r="G1" s="14"/>
       <c r="H1" s="14"/>
     </row>
-    <row r="2" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
@@ -1134,7 +1134,7 @@
       <c r="G2" s="17"/>
       <c r="H2" s="17"/>
     </row>
-    <row r="3" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="19"/>
       <c r="B3" s="20"/>
       <c r="C3" s="20"/>
@@ -1144,7 +1144,7 @@
       <c r="G3" s="20"/>
       <c r="H3" s="20"/>
     </row>
-    <row r="4" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="19"/>
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
@@ -1154,7 +1154,7 @@
       <c r="G4" s="20"/>
       <c r="H4" s="20"/>
     </row>
-    <row r="5" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
       <c r="B5" s="23"/>
       <c r="C5" s="23"/>
@@ -1164,7 +1164,7 @@
       <c r="G5" s="23"/>
       <c r="H5" s="23"/>
     </row>
-    <row r="6" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3" t="s">
         <v>11</v>
@@ -1208,7 +1208,7 @@
       <c r="G7" s="6"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3" t="s">
         <v>11</v>
@@ -1226,7 +1226,7 @@
       <c r="G8" s="6"/>
       <c r="H8" s="8"/>
     </row>
-    <row r="9" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3" t="s">
         <v>11</v>
@@ -1250,7 +1250,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3" t="s">
         <v>11</v>
@@ -1274,7 +1274,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3" t="s">
         <v>11</v>
@@ -1298,7 +1298,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3" t="s">
         <v>11</v>
@@ -1322,7 +1322,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="3" t="s">
         <v>11</v>
@@ -1346,7 +1346,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3" t="s">
         <v>11</v>
@@ -1370,7 +1370,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3" t="s">
         <v>11</v>
@@ -1394,7 +1394,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="s">
         <v>11</v>
@@ -1418,7 +1418,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="3" t="s">
         <v>11</v>
@@ -1442,7 +1442,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="s">
         <v>11</v>
@@ -1466,7 +1466,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="3" t="s">
         <v>11</v>
@@ -1490,7 +1490,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="s">
         <v>11</v>
@@ -1514,7 +1514,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="s">
         <v>11</v>
@@ -1538,7 +1538,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
         <v>11</v>
@@ -1562,7 +1562,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
         <v>11</v>
@@ -1586,7 +1586,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3" t="s">
         <v>11</v>
@@ -1610,7 +1610,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="3" t="s">
         <v>11</v>
@@ -1634,7 +1634,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>3</v>
       </c>
@@ -1660,7 +1660,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="3" t="s">
         <v>11</v>
@@ -1678,7 +1678,7 @@
       <c r="G27" s="6"/>
       <c r="H27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3" t="s">
         <v>11</v>
@@ -1702,7 +1702,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="3" t="s">
         <v>11</v>
@@ -1726,7 +1726,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>11</v>
@@ -1750,7 +1750,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>11</v>
@@ -1774,7 +1774,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>11</v>
@@ -1798,7 +1798,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>11</v>
@@ -1822,7 +1822,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3" t="s">
         <v>11</v>
@@ -1846,7 +1846,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>3</v>
       </c>
@@ -1872,7 +1872,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
         <v>11</v>
@@ -1890,7 +1890,7 @@
       <c r="G36" s="6"/>
       <c r="H36" s="7"/>
     </row>
-    <row r="37" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3" t="s">
         <v>11</v>
@@ -1914,7 +1914,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3" t="s">
         <v>11</v>
@@ -1938,7 +1938,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3" t="s">
         <v>11</v>
@@ -1962,7 +1962,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3" t="s">
         <v>11</v>
@@ -1986,7 +1986,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="3" t="s">
         <v>11</v>
@@ -2010,7 +2010,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="3" t="s">
         <v>11</v>
@@ -2034,7 +2034,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3" t="s">
         <v>11</v>
@@ -2058,7 +2058,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>3</v>
       </c>
@@ -2084,7 +2084,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="3" t="s">
         <v>11</v>
@@ -2104,7 +2104,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="3" t="s">
         <v>11</v>
@@ -2128,7 +2128,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="3" t="s">
         <v>11</v>
@@ -2152,7 +2152,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3" t="s">
         <v>11</v>
@@ -2176,7 +2176,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>3</v>
       </c>
@@ -2202,7 +2202,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="3" t="s">
         <v>11</v>
@@ -2222,7 +2222,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3" t="s">
         <v>11</v>
@@ -2246,7 +2246,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="3" t="s">
         <v>11</v>
@@ -2270,7 +2270,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>3</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
       <c r="B54" s="3" t="s">
         <v>11</v>
@@ -2316,7 +2316,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3" t="s">
         <v>11</v>
@@ -2340,7 +2340,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3" t="s">
         <v>11</v>
@@ -2364,7 +2364,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>3</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
         <v>11</v>
@@ -2408,7 +2408,7 @@
       <c r="G58" s="6"/>
       <c r="H58" s="8"/>
     </row>
-    <row r="59" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
       <c r="B59" s="3" t="s">
         <v>11</v>

</xml_diff>